<commit_message>
docs(report): chuyen cac muc GitHub sang Week 2 va giu Week 1 ve 9 muc chuan
</commit_message>
<xml_diff>
--- a/PRJ301_SE20C_Group 7.xlsx
+++ b/PRJ301_SE20C_Group 7.xlsx
@@ -946,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1445,138 +1445,9 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="80" customHeight="1">
-      <c r="A11" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="24" t="inlineStr">
-        <is>
-          <t>Requirement &amp; Analysis</t>
-        </is>
-      </c>
-      <c r="C11" s="24" t="inlineStr">
-        <is>
-          <t>Analyze AITA project structure and Servlet-DAO-JSP request flow</t>
-        </is>
-      </c>
-      <c r="D11" s="24" t="inlineStr">
-        <is>
-          <t>ChatGPT</t>
-        </is>
-      </c>
-      <c r="E11" s="24" t="inlineStr">
-        <is>
-          <t>Explained the project architecture, including Browser → Tomcat → Servlet → DAO → SQL Server → JSP flow; identified the responsibilities of controllers, DAOs, models, services and filters.</t>
-        </is>
-      </c>
-      <c r="F11" s="24" t="inlineStr">
-        <is>
-          <t>Cross-checked the explanation with the existing project folders and source files. Distinguished implemented modules from static preview pages.</t>
-        </is>
-      </c>
-      <c r="G11" s="25" t="n"/>
-      <c r="H11" s="24" t="inlineStr">
-        <is>
-          <t>7 main source layers analyzed; 6 Servlet controllers identified</t>
-        </is>
-      </c>
-      <c r="I11" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="J11" s="24" t="inlineStr">
-        <is>
-          <t>AI explanation depends on the current source code and may not reflect future changes unless the project is reviewed againAI explanation depends on the current source code and may not reflect future changes unless the project is reviewed again</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="80" customHeight="1">
-      <c r="A12" s="23" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="24" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="C12" s="24" t="inlineStr">
-        <is>
-          <t>Define Admin role in the ERD and system workflow</t>
-        </is>
-      </c>
-      <c r="D12" s="24" t="inlineStr">
-        <is>
-          <t>ChatGPT</t>
-        </is>
-      </c>
-      <c r="E12" s="24" t="inlineStr">
-        <is>
-          <t>Recommended modeling Admin as a role value in the existing Users entity instead of creating a separate Admin table. Defined administrative responsibilities for user management, configuration, report monitoring, appeal handling and audit review.</t>
-        </is>
-      </c>
-      <c r="F12" s="24" t="inlineStr">
-        <is>
-          <t>Compared the role design with current Users table usage and selected Users.role = ADMIN as the simpler design for this project.</t>
-        </is>
-      </c>
-      <c r="G12" s="25" t="n"/>
-      <c r="H12" s="24" t="inlineStr">
-        <is>
-          <t>1 role design decision; 6 admin responsibilities defined</t>
-        </is>
-      </c>
-      <c r="I12" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="J12" s="24" t="inlineStr">
-        <is>
-          <t>Role values alone cannot enforce all permissions; access control must also be checked in Servlet/filter logic.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="80" customHeight="1">
-      <c r="A13" s="23" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="24" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-      <c r="C13" s="24" t="inlineStr">
-        <is>
-          <t>Refine future ERD entities for plagiarism detection workflow</t>
-        </is>
-      </c>
-      <c r="D13" s="24" t="inlineStr">
-        <is>
-          <t>ChatGPT</t>
-        </is>
-      </c>
-      <c r="E13" s="24" t="inlineStr">
-        <is>
-          <t>Extracted candidate entities from the business description, filtered them by relevance, and proposed core additions: CourseStudents, SubmissionFiles, ScanJobs, Appeals, DetectionSettings and AuditLogs.</t>
-        </is>
-      </c>
-      <c r="F13" s="24" t="inlineStr">
-        <is>
-          <t>Retained only entities directly supporting course enrollment, file submission, plagiarism scanning, reporting and appeals. Avoided adding unnecessary entities outside the project scope.</t>
-        </is>
-      </c>
-      <c r="G13" s="25" t="n"/>
-      <c r="H13" s="24" t="inlineStr">
-        <is>
-          <t>16 candidate entities identified; 6 future entities recommended</t>
-        </is>
-      </c>
-      <c r="I13" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="J13" s="24" t="inlineStr">
-        <is>
-          <t>Adding too many entities early can make the database overly complex; the team must implement only features included in the final scope.</t>
-        </is>
-      </c>
-    </row>
+    <row r="11" ht="80" customHeight="1"/>
+    <row r="12" ht="80" customHeight="1"/>
+    <row r="13" ht="80" customHeight="1"/>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
@@ -1594,7 +1465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1754,6 +1625,138 @@
       <c r="J3" s="27" t="inlineStr">
         <is>
           <t>AI initially pushed towards enterprise overengineering (Class Table Inheritance) which would introduce multi-table JOIN overhead and connection management risks in raw JDBC servlets without an ORM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="90" customHeight="1">
+      <c r="A4" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t>Requirement &amp; Analysis</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>Analyze AITA project structure and Servlet-DAO-JSP request flow</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>Explained the project architecture, including Browser → Tomcat → Servlet → DAO → SQL Server → JSP flow; identified the responsibilities of controllers, DAOs, models, services and filters.</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>Cross-checked the explanation with the existing project folders and source files. Distinguished implemented modules from static preview pages.</t>
+        </is>
+      </c>
+      <c r="G4" s="27" t="n"/>
+      <c r="H4" s="27" t="inlineStr">
+        <is>
+          <t>7 main source layers analyzed; 6 Servlet controllers identified</t>
+        </is>
+      </c>
+      <c r="I4" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" s="27" t="inlineStr">
+        <is>
+          <t>AI explanation depends on the current source code and may not reflect future changes unless the project is reviewed again</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="90" customHeight="1">
+      <c r="A5" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="27" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="inlineStr">
+        <is>
+          <t>Define Admin role in the ERD and system workflow</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>Recommended modeling Admin as a role value in the existing Users entity instead of creating a separate Admin table. Defined administrative responsibilities for user management, configuration, report monitoring, appeal handling and audit review.</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>Compared the role design with current Users table usage and selected Users.role = ADMIN as the simpler design for this project.</t>
+        </is>
+      </c>
+      <c r="G5" s="27" t="n"/>
+      <c r="H5" s="27" t="inlineStr">
+        <is>
+          <t>1 role design decision; 6 admin responsibilities defined</t>
+        </is>
+      </c>
+      <c r="I5" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" s="27" t="inlineStr">
+        <is>
+          <t>Role values alone cannot enforce all permissions; access control must also be checked in Servlet/filter logic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>Refine future ERD entities for plagiarism detection workflow</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>Extracted candidate entities from the business description, filtered them by relevance, and proposed core additions: CourseStudents, SubmissionFiles, ScanJobs, Appeals, DetectionSettings and AuditLogs.</t>
+        </is>
+      </c>
+      <c r="F6" s="27" t="inlineStr">
+        <is>
+          <t>Retained only entities directly supporting course enrollment, file submission, plagiarism scanning, reporting and appeals. Avoided adding unnecessary entities outside the project scope.</t>
+        </is>
+      </c>
+      <c r="G6" s="27" t="n"/>
+      <c r="H6" s="27" t="inlineStr">
+        <is>
+          <t>16 candidate entities identified; 6 future entities recommended</t>
+        </is>
+      </c>
+      <c r="I6" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" s="27" t="inlineStr">
+        <is>
+          <t>Adding too many entities early can make the database overly complex; the team must implement only features included in the final scope.</t>
         </is>
       </c>
     </row>

</xml_diff>